<commit_message>
Train and testing of the module
</commit_message>
<xml_diff>
--- a/All_Runs_Summary_Polyp.xlsx
+++ b/All_Runs_Summary_Polyp.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,10 +481,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A2" t="n">
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -518,6 +516,46 @@
       </c>
       <c r="J2" t="n">
         <v>8.172754838709677</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MK_UNet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ClinicDB</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9299816412310447</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8725009204879883</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9424032258064515</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.994083870967742</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.9223112903225805</v>
+      </c>
+      <c r="J3" t="n">
+        <v>15.06378548387097</v>
       </c>
     </row>
   </sheetData>

</xml_diff>